<commit_message>
vault backup: 2026-07-17 16:50:23
</commit_message>
<xml_diff>
--- a/10_Projects/资产收入汇总表new.xlsx
+++ b/10_Projects/资产收入汇总表new.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr defaultThemeVersion="166925"/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -17,7 +17,7 @@
     <sheet name="Creekside Hills" sheetId="9" r:id="rId12"/>
     <sheet name="Harvest Cash Flow Budget 2025" sheetId="10" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -5770,7 +5770,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="SY Cash Flow Budget for 2026FY">
     <tabColor rgb="FFFFFFFF"/>
   </sheetPr>
@@ -6481,7 +6481,10 @@
         <f>=M14</f>
         <v>2976.5</v>
       </c>
-      <c r="P14" s="129" t="s"/>
+      <c r="P14" s="129">
+        <f>N14</f>
+        <v>3019.95</v>
+      </c>
       <c r="Q14" s="126">
         <f>=O14</f>
         <v>2976.5</v>

</xml_diff>

<commit_message>
vault backup: 2026-07-17 17:22:01
</commit_message>
<xml_diff>
--- a/10_Projects/资产收入汇总表new.xlsx
+++ b/10_Projects/资产收入汇总表new.xlsx
@@ -5032,11 +5032,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Creekside Hills 2026FY">
     <tabColor rgb="FFFFFFFF"/>
   </sheetPr>
-  <dimension ref="O30"/>
+  <dimension ref="P30"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -5081,6 +5081,11 @@
       </c>
       <c r="O1" s="32" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -5195,6 +5200,11 @@
       <c r="O5" s="44">
         <f>=SUM(C5:N5)</f>
         <v>144430</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3.00% rent uplift effective 1 Mar 2026 (A$11,916.67 -&gt; A$12,274.17/month)</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -5604,17 +5614,27 @@
       <c r="I24" s="39" t="s"/>
       <c r="J24" s="39" t="s"/>
       <c r="K24" s="46">
-        <v>28000</v>
+        <v>17771.12</v>
       </c>
       <c r="L24" s="49" t="s"/>
       <c r="M24" s="49" t="s"/>
       <c r="N24" s="49" t="s"/>
       <c r="O24" s="44">
-        <v>28000</v>
+        <f>SUM(C24:N24)</f>
+        <v>17771.12</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Main cost: Insurance A$17,771.12</t>
+        </is>
       </c>
     </row>
     <row r="25" spans="1:15">
-      <c r="A25" s="38" t="s"/>
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>Asset maintenance</t>
+        </is>
+      </c>
       <c r="B25" s="39" t="s"/>
       <c r="C25" s="39" t="s"/>
       <c r="D25" s="39" t="s"/>
@@ -5628,7 +5648,14 @@
       <c r="L25" s="40" t="s"/>
       <c r="M25" s="40" t="s"/>
       <c r="N25" s="40" t="s"/>
-      <c r="O25" s="41" t="s"/>
+      <c r="O25" s="41">
+        <v>0</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="33" t="s">
@@ -5693,19 +5720,63 @@
         <v>27</v>
       </c>
       <c r="B27" s="34" t="s"/>
-      <c r="C27" s="35" t="s"/>
-      <c r="D27" s="35" t="s"/>
-      <c r="E27" s="35" t="s"/>
-      <c r="F27" s="35" t="s"/>
-      <c r="G27" s="35" t="s"/>
-      <c r="H27" s="35" t="s"/>
-      <c r="I27" s="35" t="s"/>
-      <c r="J27" s="35" t="s"/>
-      <c r="K27" s="35" t="s"/>
-      <c r="L27" s="36" t="s"/>
-      <c r="M27" s="36" t="s"/>
-      <c r="N27" s="36" t="s"/>
-      <c r="O27" s="50" t="s"/>
+      <c r="C27" s="35">
+        <f>SUM(C21:C26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="D27" s="35">
+        <f>SUM(D21:D26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="E27" s="35">
+        <f>SUM(E21:E26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="F27" s="35">
+        <f>SUM(F21:F26)</f>
+        <v>1973.33333333333</v>
+      </c>
+      <c r="G27" s="35">
+        <f>SUM(G21:G26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="H27" s="35">
+        <f>SUM(H21:H26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="I27" s="35">
+        <f>SUM(I21:I26)</f>
+        <v>1093.33333333333</v>
+      </c>
+      <c r="J27" s="35">
+        <f>SUM(J21:J26)</f>
+        <v>1973.33333333333</v>
+      </c>
+      <c r="K27" s="35">
+        <f>SUM(K21:K26)</f>
+        <v>18896.9533333333</v>
+      </c>
+      <c r="L27" s="36">
+        <f>SUM(L21:L26)</f>
+        <v>1125.83333333333</v>
+      </c>
+      <c r="M27" s="36">
+        <f>SUM(M21:M26)</f>
+        <v>1125.83333333333</v>
+      </c>
+      <c r="N27" s="36">
+        <f>SUM(N21:N26)</f>
+        <v>2005.83333333333</v>
+      </c>
+      <c r="O27" s="50">
+        <f>SUM(O21:O26)</f>
+        <v>33661.12</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Other minor fees retained; focus on insurance and rent step-up</t>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="48" t="s"/>
@@ -5762,10 +5833,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId3"/>
-    <hyperlink ref="A6" r:id="rId4"/>
+    <hyperlink ref="B5" ns1:id="rId3"/>
+    <hyperlink ref="A6" ns1:id="rId4"/>
   </hyperlinks>
-  <legacyDrawing r:id="rId0"/>
+  <legacyDrawing ns1:id="rId0"/>
 </worksheet>
 </file>
 

</xml_diff>